<commit_message>
setup function change, experiment error
</commit_message>
<xml_diff>
--- a/bigresults/results.xlsx
+++ b/bigresults/results.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -504,331 +504,390 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Load Peak</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>280</v>
+      </c>
+      <c r="I2" t="n">
+        <v>666.2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Load Peak</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>MEAN</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="C3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>280</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>666.2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Load Peak</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>STDEV</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="C4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Load Avg</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B6" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C6" t="n">
         <v>5.9</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="H6" t="n">
+        <v>278.7</v>
+      </c>
+      <c r="I6" t="n">
+        <v>843.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Load Avg</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>MEAN</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>278.7</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>843.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Load Avg</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>STDEV</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>No Mig</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>6</v>
+      </c>
+      <c r="E10" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G10" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>525.9</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1535.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>No Mig</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>MEAN</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>525.9</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>1535.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>No Mig</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>STDEV</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Tardis</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="D14" t="n">
         <v>6.1</v>
       </c>
-      <c r="E5" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="F5" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="G5" t="n">
-        <v>44</v>
-      </c>
-      <c r="H5" t="n">
-        <v>285.6</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1451.1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Load Avg</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="E14" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F14" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="G14" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="H14" t="n">
+        <v>282.1</v>
+      </c>
+      <c r="I14" t="n">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Tardis</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>MEAN</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C15" s="2" t="n">
         <v>5.9</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D15" s="2" t="n">
         <v>6.1</v>
       </c>
-      <c r="E6" s="2" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>285.6</v>
-      </c>
-      <c r="I6" s="2" t="n">
-        <v>1451.1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Load Avg</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="E15" s="2" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>282.1</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Tardis</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>STDEV</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>No Mig</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C9" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="D9" t="n">
-        <v>6</v>
-      </c>
-      <c r="E9" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="F9" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="G9" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="H9" t="n">
-        <v>564.1</v>
-      </c>
-      <c r="I9" t="n">
-        <v>1497.7</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>No Mig</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>MEAN</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="D10" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="2" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>42.9</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>564.1</v>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>1497.7</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>No Mig</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>STDEV</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Tardis</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="D13" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="E13" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="F13" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="G13" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="H13" t="n">
-        <v>292.2</v>
-      </c>
-      <c r="I13" t="n">
-        <v>918.3</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Tardis</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>MEAN</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>13.2</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>292.2</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>918.3</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Tardis</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>STDEV</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" s="3" t="n">
+      <c r="C16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -947,6 +1006,48 @@
           <t>Load Peak</t>
         </is>
       </c>
+      <c r="B2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>280</v>
+      </c>
+      <c r="H2" t="n">
+        <v>666.2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -958,22 +1059,22 @@
         <v>5.9</v>
       </c>
       <c r="C3" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="D3" t="n">
-        <v>6.5</v>
+        <v>7.1</v>
       </c>
       <c r="E3" t="n">
-        <v>11.2</v>
+        <v>13.4</v>
       </c>
       <c r="F3" t="n">
-        <v>44</v>
+        <v>43.7</v>
       </c>
       <c r="G3" t="n">
-        <v>285.6</v>
+        <v>278.7</v>
       </c>
       <c r="H3" t="n">
-        <v>1451.1</v>
+        <v>843.5</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -1010,19 +1111,19 @@
         <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
       <c r="E4" t="n">
-        <v>8.199999999999999</v>
+        <v>7.2</v>
       </c>
       <c r="F4" t="n">
-        <v>42.9</v>
+        <v>41.3</v>
       </c>
       <c r="G4" t="n">
-        <v>564.1</v>
+        <v>525.9</v>
       </c>
       <c r="H4" t="n">
-        <v>1497.7</v>
+        <v>1535.5</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -1062,16 +1163,16 @@
         <v>7.1</v>
       </c>
       <c r="E5" t="n">
-        <v>13.2</v>
+        <v>14.2</v>
       </c>
       <c r="F5" t="n">
-        <v>44.9</v>
+        <v>43.6</v>
       </c>
       <c r="G5" t="n">
-        <v>292.2</v>
+        <v>282.1</v>
       </c>
       <c r="H5" t="n">
-        <v>918.3</v>
+        <v>823</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>

</xml_diff>